<commit_message>
Migrate Contact Us and Apply for Credit; add embed-app block
embed-app embeds an application started by a form POST into an iframe
(Apply for Credit's credit application). Importer: Contact Us moves to the
content-page template with a validated columns-callout parser; new
apply-for-credit template, embed-app parser and import script; cleanup drops
empty lists, sr-only skip links and the credit app loader; both pages added
to the migrated-pages link map.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="266">
   <si>
     <t>_reportFile</t>
   </si>
@@ -91,13 +91,34 @@
     <t>https://www.toyotafinancial.com/us/en/accessibility.html</t>
   </si>
   <si>
+    <t>us/en/contact-us.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout"]</t>
+  </si>
+  <si>
+    <t>us/en/contact-us</t>
+  </si>
+  <si>
+    <t>content-page</t>
+  </si>
+  <si>
+    <t>2026-10-04T04:59:21.156Z</t>
+  </si>
+  <si>
+    <t>Contact Us | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/contact_us.html</t>
+  </si>
+  <si>
     <t>us/en/online-policies-and-agreements.report.json</t>
   </si>
   <si>
     <t>us/en/online-policies-and-agreements</t>
   </si>
   <si>
-    <t>2026-10-03T23:57:11.653Z</t>
+    <t>2026-10-04T04:00:51.111Z</t>
   </si>
   <si>
     <t>Online Policies and Agreements | Toyota Financial</t>
@@ -115,7 +136,7 @@
     <t>us/en/online-privacy-policy</t>
   </si>
   <si>
-    <t>2026-10-03T23:57:18.617Z</t>
+    <t>2026-10-04T04:00:56.551Z</t>
   </si>
   <si>
     <t>Online Privacy Policies | Toyota Financial</t>
@@ -188,9 +209,6 @@
   </si>
   <si>
     <t>us/en/planning-tools/get-started</t>
-  </si>
-  <si>
-    <t>content-page</t>
   </si>
   <si>
     <t>2026-10-04T02:50:21.226Z</t>
@@ -1185,7 +1203,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -1295,7 +1313,7 @@
         <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
@@ -1304,30 +1322,30 @@
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
       </c>
       <c r="G4" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="J4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -1336,7 +1354,7 @@
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
         <v>14</v>
@@ -1345,21 +1363,21 @@
         <v>22</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -1368,7 +1386,7 @@
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F6" t="s">
         <v>14</v>
@@ -1377,21 +1395,21 @@
         <v>22</v>
       </c>
       <c r="H6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
@@ -1400,30 +1418,30 @@
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F7" t="s">
         <v>14</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="H7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
@@ -1502,24 +1520,24 @@
         <v>14</v>
       </c>
       <c r="G10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" t="s">
         <v>66</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>67</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>68</v>
-      </c>
-      <c r="J10" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
@@ -1534,24 +1552,24 @@
         <v>14</v>
       </c>
       <c r="G11" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
@@ -1560,30 +1578,30 @@
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F12" t="s">
         <v>14</v>
       </c>
       <c r="G12" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C13" t="s">
         <v>12</v>
@@ -1592,30 +1610,30 @@
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
@@ -1624,30 +1642,30 @@
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F14" t="s">
         <v>14</v>
       </c>
       <c r="G14" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B15" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
@@ -1656,30 +1674,30 @@
         <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F15" t="s">
         <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H15" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B16" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C16" t="s">
         <v>12</v>
@@ -1688,30 +1706,30 @@
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F16" t="s">
         <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C17" t="s">
         <v>12</v>
@@ -1720,30 +1738,30 @@
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F17" t="s">
         <v>14</v>
       </c>
       <c r="G17" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
         <v>12</v>
@@ -1752,30 +1770,30 @@
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
       </c>
       <c r="G18" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B19" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C19" t="s">
         <v>12</v>
@@ -1784,30 +1802,30 @@
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F19" t="s">
         <v>14</v>
       </c>
       <c r="G19" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B20" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C20" t="s">
         <v>12</v>
@@ -1816,30 +1834,30 @@
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
       </c>
       <c r="G20" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B21" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C21" t="s">
         <v>12</v>
@@ -1848,30 +1866,30 @@
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F21" t="s">
         <v>14</v>
       </c>
       <c r="G21" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B22" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -1880,30 +1898,30 @@
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
       </c>
       <c r="G22" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H22" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I22" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J22" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B23" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C23" t="s">
         <v>12</v>
@@ -1912,30 +1930,30 @@
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F23" t="s">
         <v>14</v>
       </c>
       <c r="G23" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H23" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I23" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J23" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B24" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
@@ -1944,30 +1962,30 @@
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F24" t="s">
         <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H24" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I24" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J24" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B25" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C25" t="s">
         <v>12</v>
@@ -1976,30 +1994,30 @@
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F25" t="s">
         <v>14</v>
       </c>
       <c r="G25" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H25" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I25" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J25" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B26" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
@@ -2008,30 +2026,30 @@
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F26" t="s">
         <v>14</v>
       </c>
       <c r="G26" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H26" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I26" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J26" t="s">
-        <v>48</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C27" t="s">
         <v>12</v>
@@ -2040,30 +2058,30 @@
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F27" t="s">
         <v>14</v>
       </c>
       <c r="G27" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H27" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I27" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="J27" t="s">
-        <v>153</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B28" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C28" t="s">
         <v>12</v>
@@ -2072,30 +2090,30 @@
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F28" t="s">
         <v>14</v>
       </c>
       <c r="G28" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H28" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I28" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B29" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C29" t="s">
         <v>12</v>
@@ -2104,30 +2122,30 @@
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F29" t="s">
         <v>14</v>
       </c>
       <c r="G29" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H29" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I29" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J29" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C30" t="s">
         <v>12</v>
@@ -2136,30 +2154,30 @@
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F30" t="s">
         <v>14</v>
       </c>
       <c r="G30" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H30" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I30" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J30" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C31" t="s">
         <v>12</v>
@@ -2168,30 +2186,30 @@
         <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F31" t="s">
         <v>14</v>
       </c>
       <c r="G31" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H31" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I31" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J31" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B32" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
@@ -2200,30 +2218,30 @@
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F32" t="s">
         <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H32" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I32" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J32" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B33" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C33" t="s">
         <v>12</v>
@@ -2232,30 +2250,30 @@
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F33" t="s">
         <v>14</v>
       </c>
       <c r="G33" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H33" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I33" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J33" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B34" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C34" t="s">
         <v>12</v>
@@ -2264,30 +2282,30 @@
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F34" t="s">
         <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H34" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I34" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J34" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B35" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C35" t="s">
         <v>12</v>
@@ -2296,30 +2314,30 @@
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F35" t="s">
         <v>14</v>
       </c>
       <c r="G35" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H35" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I35" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J35" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B36" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C36" t="s">
         <v>12</v>
@@ -2328,30 +2346,30 @@
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F36" t="s">
         <v>14</v>
       </c>
       <c r="G36" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H36" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I36" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J36" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B37" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C37" t="s">
         <v>12</v>
@@ -2360,30 +2378,30 @@
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F37" t="s">
         <v>14</v>
       </c>
       <c r="G37" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H37" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I37" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J37" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B38" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C38" t="s">
         <v>12</v>
@@ -2392,30 +2410,30 @@
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F38" t="s">
         <v>14</v>
       </c>
       <c r="G38" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H38" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I38" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J38" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B39" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C39" t="s">
         <v>12</v>
@@ -2424,30 +2442,30 @@
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F39" t="s">
         <v>14</v>
       </c>
       <c r="G39" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H39" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I39" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J39" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B40" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C40" t="s">
         <v>12</v>
@@ -2456,30 +2474,30 @@
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F40" t="s">
         <v>14</v>
       </c>
       <c r="G40" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H40" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="I40" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J40" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B41" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C41" t="s">
         <v>12</v>
@@ -2488,30 +2506,30 @@
         <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F41" t="s">
         <v>14</v>
       </c>
       <c r="G41" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H41" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="I41" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J41" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B42" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C42" t="s">
         <v>12</v>
@@ -2520,30 +2538,30 @@
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F42" t="s">
         <v>14</v>
       </c>
       <c r="G42" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H42" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="I42" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="J42" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B43" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C43" t="s">
         <v>12</v>
@@ -2552,30 +2570,30 @@
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F43" t="s">
         <v>14</v>
       </c>
       <c r="G43" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H43" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="I43" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J43" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B44" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C44" t="s">
         <v>12</v>
@@ -2584,30 +2602,30 @@
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F44" t="s">
         <v>14</v>
       </c>
       <c r="G44" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H44" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I44" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J44" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B45" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C45" t="s">
         <v>12</v>
@@ -2616,30 +2634,30 @@
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F45" t="s">
         <v>14</v>
       </c>
       <c r="G45" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H45" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="I45" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="J45" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B46" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C46" t="s">
         <v>12</v>
@@ -2648,30 +2666,30 @@
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F46" t="s">
         <v>14</v>
       </c>
       <c r="G46" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H46" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="I46" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J46" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B47" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C47" t="s">
         <v>12</v>
@@ -2680,54 +2698,86 @@
         <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F47" t="s">
         <v>14</v>
       </c>
       <c r="G47" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H47" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="I47" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J47" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B48" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="C48" t="s">
-        <v>255</v>
+        <v>12</v>
       </c>
       <c r="D48" t="s">
+        <v>12</v>
+      </c>
+      <c r="E48" t="s">
         <v>256</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
+        <v>14</v>
+      </c>
+      <c r="G48" t="s">
+        <v>72</v>
+      </c>
+      <c r="H48" t="s">
         <v>257</v>
       </c>
-      <c r="F48" t="s">
+      <c r="I48" t="s">
         <v>258</v>
       </c>
-      <c r="G48" t="s">
-        <v>12</v>
-      </c>
-      <c r="H48" t="s">
+      <c r="J48" t="s">
         <v>259</v>
       </c>
-      <c r="I48" t="s">
-        <v>12</v>
-      </c>
-      <c r="J48" t="s">
-        <v>69</v>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>260</v>
+      </c>
+      <c r="B49" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49" t="s">
+        <v>261</v>
+      </c>
+      <c r="D49" t="s">
+        <v>262</v>
+      </c>
+      <c r="E49" t="s">
+        <v>263</v>
+      </c>
+      <c r="F49" t="s">
+        <v>264</v>
+      </c>
+      <c r="G49" t="s">
+        <v>12</v>
+      </c>
+      <c r="H49" t="s">
+        <v>265</v>
+      </c>
+      <c r="I49" t="s">
+        <v>12</v>
+      </c>
+      <c r="J49" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Importer: validated content-page parsers, 15-page content batch
Validated/fixed the content-page parsers (table-caption, tabs-plans,
columns-card blog index); all 10 registered in import-content-page.js with
tabs-plans last; 28 requested pages added to the migrated-pages link map.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="356">
   <si>
     <t>_reportFile</t>
   </si>
@@ -145,6 +145,24 @@
     <t>https://www.toyotafinancial.com/us/en/online_privacy_policy.html</t>
   </si>
   <si>
+    <t>us/en/tfs-thoughtfuel-blog.report.json</t>
+  </si>
+  <si>
+    <t>["columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card","columns-card"]</t>
+  </si>
+  <si>
+    <t>us/en/tfs-thoughtfuel-blog</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:06:26.543Z</t>
+  </si>
+  <si>
+    <t>TFS ThoughtFuel Blog | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/TFS_ThoughtFuel_Blog.html</t>
+  </si>
+  <si>
     <t>us/en/about-us/company-overview.report.json</t>
   </si>
   <si>
@@ -163,6 +181,60 @@
     <t>https://www.toyotafinancial.com/us/en/about_us/company_overview.html</t>
   </si>
   <si>
+    <t>us/en/financing-options/buy-a-toyota.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","columns-callout","columns-callout","accordion-faq"]</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/buy-a-toyota</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:04:38.180Z</t>
+  </si>
+  <si>
+    <t>Buy a Toyota | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/buy_a_toyota.html</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/leasing-a-toyota.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","columns-callout","columns-callout","accordion-faq","accordion-faq"]</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/leasing-a-toyota</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:04:43.836Z</t>
+  </si>
+  <si>
+    <t>Lease a Toyota | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/leasing_a_toyota.html</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/toyota-rewards-visa.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","columns-callout"]</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/toyota-rewards-visa</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:06:21.243Z</t>
+  </si>
+  <si>
+    <t>Toyota Rewards Visa | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/toyota_rewards_visa.html</t>
+  </si>
+  <si>
     <t>us/en/fragments/faq-help.report.json</t>
   </si>
   <si>
@@ -181,6 +253,27 @@
     <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/Guaranteed_Auto_Protection_GAP.html</t>
   </si>
   <si>
+    <t>us/en/planning-tools/apply-for-credit.report.json</t>
+  </si>
+  <si>
+    <t>["embed-app"]</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/apply-for-credit</t>
+  </si>
+  <si>
+    <t>apply-for-credit</t>
+  </si>
+  <si>
+    <t>2026-10-04T05:05:55.110Z</t>
+  </si>
+  <si>
+    <t>Apply for Credit | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/apply_for_credit.html</t>
+  </si>
+  <si>
     <t>us/en/planning-tools/faq.report.json</t>
   </si>
   <si>
@@ -220,6 +313,192 @@
     <t>https://www.toyotafinancial.com/us/en/planning_tools/get_started.html</t>
   </si>
   <si>
+    <t>us/en/planning-tools/ways-to-pay.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","accordion-boxed","accordion-boxed","accordion-boxed","accordion-boxed","accordion-boxed","accordion-boxed","accordion-boxed"]</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/ways-to-pay</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:04:33.230Z</t>
+  </si>
+  <si>
+    <t>Ways to Pay | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/ways_to_pay.html</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/guaranteed-auto-protection.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","columns-callout","video-poster"]</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/guaranteed-auto-protection</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:03:13.602Z</t>
+  </si>
+  <si>
+    <t>Guaranteed Auto Protection | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/vehicle_protection_plan/guaranteed_auto_protection.html</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/prepaid-maintenance-plan.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","video-poster","table-caption","table-caption","table-caption","table-caption","table-caption","table-caption","table-caption","tabs-plans","tabs-plans","tabs-plans"]</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/prepaid-maintenance-plan</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:03:19.009Z</t>
+  </si>
+  <si>
+    <t>Prepaid Maintenance Plans | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/vehicle_protection_plan/prepaid_maintenance_plan.html</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/tire-wheel-protection.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","accordion-faq","accordion-faq","accordion-faq","video-poster","table-caption","table-caption","tabs-plans"]</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/tire-wheel-protection</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:03:26.503Z</t>
+  </si>
+  <si>
+    <t>Tire &amp; Wheel Protection | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/vehicle_protection_plan/tire_wheel_protection.html</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/vehicle-service-agreements.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","columns-callout","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","accordion-faq","video-poster","tabs-plans","tabs-plans","tabs-plans","tabs-plans","tabs-plans"]</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/vehicle-service-agreements</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:03:04.477Z</t>
+  </si>
+  <si>
+    <t>Vehicle Service Agreements | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/vehicle_protection_plan/vehicle_service_agreements.html</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/which-plan-is-right-for-me.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","video-poster","quiz-plans","carousel-cards"]</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/which-plan-is-right-for-me</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:02:57.966Z</t>
+  </si>
+  <si>
+    <t>Which plan is right for me? | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/vehicle_protection_plan/which_plan_is_right_for_me.html</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/for-businesses/business-solutions.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","accordion-faq"]</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/for-businesses/business-solutions</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:06:16.167Z</t>
+  </si>
+  <si>
+    <t>Business Solutions | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/for_businesses/business_solutions.html</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/rebate-finance-programs/find-rebate-finance-programs.report.json</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/rebate-finance-programs/find-rebate-finance-programs</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:04:51.364Z</t>
+  </si>
+  <si>
+    <t>Find a Program | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/rebate_finance_programs/find_rebate_finance_programs.html</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/rebate-finance-programs/repeat-customers.report.json</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/rebate-finance-programs/repeat-customers</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:04:57.928Z</t>
+  </si>
+  <si>
+    <t>Repeat Customers | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/rebate_finance_programs/repeat_customers.html</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/understanding-credit/credit-101.report.json</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/understanding-credit/credit-101</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:06:04.024Z</t>
+  </si>
+  <si>
+    <t>Credit 101 | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/understanding_credit/credit_101.html</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/understanding-credit/credit-tips.report.json</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/understanding-credit/credit-tips</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:06:09.456Z</t>
+  </si>
+  <si>
+    <t>Credit Tips | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/understanding_credit/credit_tips.html</t>
+  </si>
+  <si>
     <t>us/en/planning-tools/faq/about-credit.report.json</t>
   </si>
   <si>
@@ -340,9 +619,6 @@
     <t>2026-10-03T23:52:08.098Z</t>
   </si>
   <si>
-    <t>Business Solutions | Toyota Financial</t>
-  </si>
-  <si>
     <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/business_solutions.html</t>
   </si>
   <si>
@@ -445,9 +721,6 @@
     <t>2026-10-03T23:54:35.448Z</t>
   </si>
   <si>
-    <t>Vehicle Service Agreements | Toyota Financial</t>
-  </si>
-  <si>
     <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/financing_and_protection_products.html</t>
   </si>
   <si>
@@ -710,9 +983,6 @@
   </si>
   <si>
     <t>2026-10-03T23:54:14.842Z</t>
-  </si>
-  <si>
-    <t>Repeat Customers | Toyota Financial</t>
   </si>
   <si>
     <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/repeat_customers.html</t>
@@ -1203,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -1424,7 +1694,7 @@
         <v>14</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H7" t="s">
         <v>47</v>
@@ -1441,7 +1711,7 @@
         <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
@@ -1450,13 +1720,13 @@
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F8" t="s">
         <v>14</v>
       </c>
       <c r="G8" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="H8" t="s">
         <v>53</v>
@@ -1488,33 +1758,33 @@
         <v>14</v>
       </c>
       <c r="G9" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" t="s">
         <v>59</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>60</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>61</v>
-      </c>
-      <c r="J9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" t="s">
         <v>63</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
         <v>64</v>
-      </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" t="s">
-        <v>65</v>
       </c>
       <c r="F10" t="s">
         <v>14</v>
@@ -1523,85 +1793,85 @@
         <v>29</v>
       </c>
       <c r="H10" t="s">
+        <v>65</v>
+      </c>
+      <c r="I10" t="s">
         <v>66</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>67</v>
-      </c>
-      <c r="J10" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" t="s">
         <v>69</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
         <v>70</v>
       </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" t="s">
         <v>71</v>
       </c>
-      <c r="F11" t="s">
-        <v>14</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="I11" t="s">
         <v>72</v>
       </c>
-      <c r="H11" t="s">
+      <c r="J11" t="s">
         <v>73</v>
-      </c>
-      <c r="I11" t="s">
-        <v>74</v>
-      </c>
-      <c r="J11" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
         <v>76</v>
       </c>
-      <c r="B12" t="s">
-        <v>70</v>
-      </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="H12" t="s">
         <v>77</v>
       </c>
-      <c r="F12" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" t="s">
-        <v>72</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>78</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>79</v>
-      </c>
-      <c r="J12" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" t="s">
         <v>81</v>
-      </c>
-      <c r="B13" t="s">
-        <v>70</v>
       </c>
       <c r="C13" t="s">
         <v>12</v>
@@ -1616,24 +1886,24 @@
         <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="H13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
@@ -1642,30 +1912,30 @@
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F14" t="s">
         <v>14</v>
       </c>
       <c r="G14" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="H14" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="I14" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="J14" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
@@ -1674,30 +1944,30 @@
         <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F15" t="s">
         <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H15" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I15" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="J15" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="C16" t="s">
         <v>12</v>
@@ -1706,30 +1976,30 @@
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F16" t="s">
         <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H16" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="I16" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="J16" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>107</v>
       </c>
       <c r="C17" t="s">
         <v>12</v>
@@ -1738,30 +2008,30 @@
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="F17" t="s">
         <v>14</v>
       </c>
       <c r="G17" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H17" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="I17" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="J17" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>113</v>
       </c>
       <c r="C18" t="s">
         <v>12</v>
@@ -1770,30 +2040,30 @@
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
       </c>
       <c r="G18" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H18" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="I18" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="J18" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>119</v>
       </c>
       <c r="C19" t="s">
         <v>12</v>
@@ -1802,30 +2072,30 @@
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F19" t="s">
         <v>14</v>
       </c>
       <c r="G19" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H19" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="I19" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="J19" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>125</v>
       </c>
       <c r="C20" t="s">
         <v>12</v>
@@ -1834,30 +2104,30 @@
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
       </c>
       <c r="G20" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H20" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="I20" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="J20" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>131</v>
       </c>
       <c r="C21" t="s">
         <v>12</v>
@@ -1866,30 +2136,30 @@
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="F21" t="s">
         <v>14</v>
       </c>
       <c r="G21" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H21" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="I21" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="J21" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="B22" t="s">
-        <v>70</v>
+        <v>137</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -1898,30 +2168,30 @@
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
       </c>
       <c r="G22" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H22" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="I22" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="J22" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C23" t="s">
         <v>12</v>
@@ -1930,30 +2200,30 @@
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="F23" t="s">
         <v>14</v>
       </c>
       <c r="G23" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H23" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="I23" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="J23" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
@@ -1962,30 +2232,30 @@
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="F24" t="s">
         <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H24" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="I24" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="J24" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="C25" t="s">
         <v>12</v>
@@ -1994,30 +2264,30 @@
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="F25" t="s">
         <v>14</v>
       </c>
       <c r="G25" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H25" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="I25" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="J25" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="B26" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
@@ -2026,30 +2296,30 @@
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F26" t="s">
         <v>14</v>
       </c>
       <c r="G26" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="H26" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="I26" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="J26" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="B27" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C27" t="s">
         <v>12</v>
@@ -2058,30 +2328,30 @@
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="F27" t="s">
         <v>14</v>
       </c>
       <c r="G27" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H27" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="I27" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="J27" t="s">
-        <v>55</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="B28" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C28" t="s">
         <v>12</v>
@@ -2090,30 +2360,30 @@
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="F28" t="s">
         <v>14</v>
       </c>
       <c r="G28" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H28" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="I28" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="J28" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="B29" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C29" t="s">
         <v>12</v>
@@ -2122,30 +2392,30 @@
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="F29" t="s">
         <v>14</v>
       </c>
       <c r="G29" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H29" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="I29" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="J29" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="B30" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C30" t="s">
         <v>12</v>
@@ -2154,30 +2424,30 @@
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="F30" t="s">
         <v>14</v>
       </c>
       <c r="G30" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H30" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="I30" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="J30" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="B31" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C31" t="s">
         <v>12</v>
@@ -2186,30 +2456,30 @@
         <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="F31" t="s">
         <v>14</v>
       </c>
       <c r="G31" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H31" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="I31" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="J31" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="B32" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
@@ -2218,30 +2488,30 @@
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="F32" t="s">
         <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H32" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="I32" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="J32" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="B33" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C33" t="s">
         <v>12</v>
@@ -2250,30 +2520,30 @@
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="F33" t="s">
         <v>14</v>
       </c>
       <c r="G33" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H33" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
       <c r="I33" t="s">
-        <v>183</v>
+        <v>197</v>
       </c>
       <c r="J33" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="B34" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C34" t="s">
         <v>12</v>
@@ -2282,30 +2552,30 @@
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="F34" t="s">
         <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H34" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="I34" t="s">
-        <v>188</v>
+        <v>140</v>
       </c>
       <c r="J34" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="B35" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C35" t="s">
         <v>12</v>
@@ -2314,30 +2584,30 @@
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="F35" t="s">
         <v>14</v>
       </c>
       <c r="G35" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H35" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="I35" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="J35" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="B36" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C36" t="s">
         <v>12</v>
@@ -2346,30 +2616,30 @@
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="F36" t="s">
         <v>14</v>
       </c>
       <c r="G36" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H36" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="I36" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="J36" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="B37" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C37" t="s">
         <v>12</v>
@@ -2378,30 +2648,30 @@
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="F37" t="s">
         <v>14</v>
       </c>
       <c r="G37" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H37" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="I37" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="J37" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="B38" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C38" t="s">
         <v>12</v>
@@ -2410,30 +2680,30 @@
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="F38" t="s">
         <v>14</v>
       </c>
       <c r="G38" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H38" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="I38" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="J38" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="B39" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C39" t="s">
         <v>12</v>
@@ -2442,30 +2712,30 @@
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="F39" t="s">
         <v>14</v>
       </c>
       <c r="G39" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H39" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="I39" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="J39" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="B40" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C40" t="s">
         <v>12</v>
@@ -2474,30 +2744,30 @@
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="F40" t="s">
         <v>14</v>
       </c>
       <c r="G40" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H40" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="I40" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="J40" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="B41" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C41" t="s">
         <v>12</v>
@@ -2506,30 +2776,30 @@
         <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="F41" t="s">
         <v>14</v>
       </c>
       <c r="G41" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H41" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="I41" t="s">
-        <v>223</v>
+        <v>128</v>
       </c>
       <c r="J41" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="B42" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C42" t="s">
         <v>12</v>
@@ -2538,30 +2808,30 @@
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="F42" t="s">
         <v>14</v>
       </c>
       <c r="G42" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H42" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="I42" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="J42" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="B43" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C43" t="s">
         <v>12</v>
@@ -2570,30 +2840,30 @@
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="F43" t="s">
         <v>14</v>
       </c>
       <c r="G43" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H43" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="I43" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="J43" t="s">
-        <v>234</v>
+        <v>79</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="B44" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C44" t="s">
         <v>12</v>
@@ -2602,30 +2872,30 @@
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="F44" t="s">
         <v>14</v>
       </c>
       <c r="G44" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H44" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
       <c r="I44" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="J44" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="B45" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C45" t="s">
         <v>12</v>
@@ -2634,30 +2904,30 @@
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="F45" t="s">
         <v>14</v>
       </c>
       <c r="G45" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H45" t="s">
-        <v>242</v>
+        <v>253</v>
       </c>
       <c r="I45" t="s">
-        <v>243</v>
+        <v>254</v>
       </c>
       <c r="J45" t="s">
-        <v>244</v>
+        <v>255</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>245</v>
+        <v>256</v>
       </c>
       <c r="B46" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C46" t="s">
         <v>12</v>
@@ -2666,30 +2936,30 @@
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="F46" t="s">
         <v>14</v>
       </c>
       <c r="G46" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H46" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="I46" t="s">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="J46" t="s">
-        <v>249</v>
+        <v>260</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>250</v>
+        <v>261</v>
       </c>
       <c r="B47" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C47" t="s">
         <v>12</v>
@@ -2698,30 +2968,30 @@
         <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>251</v>
+        <v>262</v>
       </c>
       <c r="F47" t="s">
         <v>14</v>
       </c>
       <c r="G47" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H47" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
       <c r="I47" t="s">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="J47" t="s">
-        <v>254</v>
+        <v>265</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="B48" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="C48" t="s">
         <v>12</v>
@@ -2730,54 +3000,566 @@
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="F48" t="s">
         <v>14</v>
       </c>
       <c r="G48" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="H48" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="I48" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
       <c r="J48" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="B49" t="s">
-        <v>12</v>
+        <v>163</v>
       </c>
       <c r="C49" t="s">
-        <v>261</v>
+        <v>12</v>
       </c>
       <c r="D49" t="s">
-        <v>262</v>
+        <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="F49" t="s">
-        <v>264</v>
+        <v>14</v>
       </c>
       <c r="G49" t="s">
-        <v>12</v>
+        <v>165</v>
       </c>
       <c r="H49" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="I49" t="s">
-        <v>12</v>
+        <v>274</v>
       </c>
       <c r="J49" t="s">
-        <v>75</v>
+        <v>275</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>276</v>
+      </c>
+      <c r="B50" t="s">
+        <v>163</v>
+      </c>
+      <c r="C50" t="s">
+        <v>12</v>
+      </c>
+      <c r="D50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" t="s">
+        <v>277</v>
+      </c>
+      <c r="F50" t="s">
+        <v>14</v>
+      </c>
+      <c r="G50" t="s">
+        <v>165</v>
+      </c>
+      <c r="H50" t="s">
+        <v>278</v>
+      </c>
+      <c r="I50" t="s">
+        <v>279</v>
+      </c>
+      <c r="J50" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>281</v>
+      </c>
+      <c r="B51" t="s">
+        <v>163</v>
+      </c>
+      <c r="C51" t="s">
+        <v>12</v>
+      </c>
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" t="s">
+        <v>282</v>
+      </c>
+      <c r="F51" t="s">
+        <v>14</v>
+      </c>
+      <c r="G51" t="s">
+        <v>165</v>
+      </c>
+      <c r="H51" t="s">
+        <v>283</v>
+      </c>
+      <c r="I51" t="s">
+        <v>284</v>
+      </c>
+      <c r="J51" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>286</v>
+      </c>
+      <c r="B52" t="s">
+        <v>163</v>
+      </c>
+      <c r="C52" t="s">
+        <v>12</v>
+      </c>
+      <c r="D52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" t="s">
+        <v>287</v>
+      </c>
+      <c r="F52" t="s">
+        <v>14</v>
+      </c>
+      <c r="G52" t="s">
+        <v>165</v>
+      </c>
+      <c r="H52" t="s">
+        <v>288</v>
+      </c>
+      <c r="I52" t="s">
+        <v>289</v>
+      </c>
+      <c r="J52" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>291</v>
+      </c>
+      <c r="B53" t="s">
+        <v>163</v>
+      </c>
+      <c r="C53" t="s">
+        <v>12</v>
+      </c>
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" t="s">
+        <v>292</v>
+      </c>
+      <c r="F53" t="s">
+        <v>14</v>
+      </c>
+      <c r="G53" t="s">
+        <v>165</v>
+      </c>
+      <c r="H53" t="s">
+        <v>293</v>
+      </c>
+      <c r="I53" t="s">
+        <v>294</v>
+      </c>
+      <c r="J53" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>296</v>
+      </c>
+      <c r="B54" t="s">
+        <v>163</v>
+      </c>
+      <c r="C54" t="s">
+        <v>12</v>
+      </c>
+      <c r="D54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" t="s">
+        <v>297</v>
+      </c>
+      <c r="F54" t="s">
+        <v>14</v>
+      </c>
+      <c r="G54" t="s">
+        <v>165</v>
+      </c>
+      <c r="H54" t="s">
+        <v>298</v>
+      </c>
+      <c r="I54" t="s">
+        <v>299</v>
+      </c>
+      <c r="J54" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>301</v>
+      </c>
+      <c r="B55" t="s">
+        <v>163</v>
+      </c>
+      <c r="C55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>302</v>
+      </c>
+      <c r="F55" t="s">
+        <v>14</v>
+      </c>
+      <c r="G55" t="s">
+        <v>165</v>
+      </c>
+      <c r="H55" t="s">
+        <v>303</v>
+      </c>
+      <c r="I55" t="s">
+        <v>304</v>
+      </c>
+      <c r="J55" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>306</v>
+      </c>
+      <c r="B56" t="s">
+        <v>163</v>
+      </c>
+      <c r="C56" t="s">
+        <v>12</v>
+      </c>
+      <c r="D56" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" t="s">
+        <v>307</v>
+      </c>
+      <c r="F56" t="s">
+        <v>14</v>
+      </c>
+      <c r="G56" t="s">
+        <v>165</v>
+      </c>
+      <c r="H56" t="s">
+        <v>308</v>
+      </c>
+      <c r="I56" t="s">
+        <v>309</v>
+      </c>
+      <c r="J56" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>311</v>
+      </c>
+      <c r="B57" t="s">
+        <v>163</v>
+      </c>
+      <c r="C57" t="s">
+        <v>12</v>
+      </c>
+      <c r="D57" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57" t="s">
+        <v>312</v>
+      </c>
+      <c r="F57" t="s">
+        <v>14</v>
+      </c>
+      <c r="G57" t="s">
+        <v>165</v>
+      </c>
+      <c r="H57" t="s">
+        <v>313</v>
+      </c>
+      <c r="I57" t="s">
+        <v>314</v>
+      </c>
+      <c r="J57" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>316</v>
+      </c>
+      <c r="B58" t="s">
+        <v>163</v>
+      </c>
+      <c r="C58" t="s">
+        <v>12</v>
+      </c>
+      <c r="D58" t="s">
+        <v>12</v>
+      </c>
+      <c r="E58" t="s">
+        <v>317</v>
+      </c>
+      <c r="F58" t="s">
+        <v>14</v>
+      </c>
+      <c r="G58" t="s">
+        <v>165</v>
+      </c>
+      <c r="H58" t="s">
+        <v>318</v>
+      </c>
+      <c r="I58" t="s">
+        <v>319</v>
+      </c>
+      <c r="J58" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>321</v>
+      </c>
+      <c r="B59" t="s">
+        <v>163</v>
+      </c>
+      <c r="C59" t="s">
+        <v>12</v>
+      </c>
+      <c r="D59" t="s">
+        <v>12</v>
+      </c>
+      <c r="E59" t="s">
+        <v>322</v>
+      </c>
+      <c r="F59" t="s">
+        <v>14</v>
+      </c>
+      <c r="G59" t="s">
+        <v>165</v>
+      </c>
+      <c r="H59" t="s">
+        <v>323</v>
+      </c>
+      <c r="I59" t="s">
+        <v>150</v>
+      </c>
+      <c r="J59" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>325</v>
+      </c>
+      <c r="B60" t="s">
+        <v>163</v>
+      </c>
+      <c r="C60" t="s">
+        <v>12</v>
+      </c>
+      <c r="D60" t="s">
+        <v>12</v>
+      </c>
+      <c r="E60" t="s">
+        <v>326</v>
+      </c>
+      <c r="F60" t="s">
+        <v>14</v>
+      </c>
+      <c r="G60" t="s">
+        <v>165</v>
+      </c>
+      <c r="H60" t="s">
+        <v>327</v>
+      </c>
+      <c r="I60" t="s">
+        <v>328</v>
+      </c>
+      <c r="J60" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>330</v>
+      </c>
+      <c r="B61" t="s">
+        <v>163</v>
+      </c>
+      <c r="C61" t="s">
+        <v>12</v>
+      </c>
+      <c r="D61" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61" t="s">
+        <v>331</v>
+      </c>
+      <c r="F61" t="s">
+        <v>14</v>
+      </c>
+      <c r="G61" t="s">
+        <v>165</v>
+      </c>
+      <c r="H61" t="s">
+        <v>332</v>
+      </c>
+      <c r="I61" t="s">
+        <v>333</v>
+      </c>
+      <c r="J61" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>335</v>
+      </c>
+      <c r="B62" t="s">
+        <v>163</v>
+      </c>
+      <c r="C62" t="s">
+        <v>12</v>
+      </c>
+      <c r="D62" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" t="s">
+        <v>336</v>
+      </c>
+      <c r="F62" t="s">
+        <v>14</v>
+      </c>
+      <c r="G62" t="s">
+        <v>165</v>
+      </c>
+      <c r="H62" t="s">
+        <v>337</v>
+      </c>
+      <c r="I62" t="s">
+        <v>338</v>
+      </c>
+      <c r="J62" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>340</v>
+      </c>
+      <c r="B63" t="s">
+        <v>163</v>
+      </c>
+      <c r="C63" t="s">
+        <v>12</v>
+      </c>
+      <c r="D63" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63" t="s">
+        <v>341</v>
+      </c>
+      <c r="F63" t="s">
+        <v>14</v>
+      </c>
+      <c r="G63" t="s">
+        <v>165</v>
+      </c>
+      <c r="H63" t="s">
+        <v>342</v>
+      </c>
+      <c r="I63" t="s">
+        <v>343</v>
+      </c>
+      <c r="J63" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>345</v>
+      </c>
+      <c r="B64" t="s">
+        <v>163</v>
+      </c>
+      <c r="C64" t="s">
+        <v>12</v>
+      </c>
+      <c r="D64" t="s">
+        <v>12</v>
+      </c>
+      <c r="E64" t="s">
+        <v>346</v>
+      </c>
+      <c r="F64" t="s">
+        <v>14</v>
+      </c>
+      <c r="G64" t="s">
+        <v>165</v>
+      </c>
+      <c r="H64" t="s">
+        <v>347</v>
+      </c>
+      <c r="I64" t="s">
+        <v>348</v>
+      </c>
+      <c r="J64" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>350</v>
+      </c>
+      <c r="B65" t="s">
+        <v>12</v>
+      </c>
+      <c r="C65" t="s">
+        <v>351</v>
+      </c>
+      <c r="D65" t="s">
+        <v>352</v>
+      </c>
+      <c r="E65" t="s">
+        <v>353</v>
+      </c>
+      <c r="F65" t="s">
+        <v>354</v>
+      </c>
+      <c r="G65" t="s">
+        <v>12</v>
+      </c>
+      <c r="H65" t="s">
+        <v>355</v>
+      </c>
+      <c r="I65" t="s">
+        <v>12</v>
+      </c>
+      <c r="J65" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add quiz-buy-lease block; How to File a Claim dropdown; 5 more content pages
quiz-buy-lease re-implements the scored Buy or Lease quiz (weights, result
rules, product cards, Start over). tabs-plans handles dropdown-only cards
(single panel per group, no tab row) for How to File a Claim. Importer:
buy-or-lease template + parser + import script; How to File a Claim, Visiting
the Dealer, College/Military Rebate and Business Credit Application move to
the content-page template.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="382">
   <si>
     <t>_reportFile</t>
   </si>
@@ -313,6 +313,21 @@
     <t>https://www.toyotafinancial.com/us/en/planning_tools/get_started.html</t>
   </si>
   <si>
+    <t>us/en/planning-tools/visiting-the-dealer.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/visiting-the-dealer</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:11:09.563Z</t>
+  </si>
+  <si>
+    <t>Visiting the Dealer | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/visiting_the_dealer.html</t>
+  </si>
+  <si>
     <t>us/en/planning-tools/ways-to-pay.report.json</t>
   </si>
   <si>
@@ -349,6 +364,24 @@
     <t>https://www.toyotafinancial.com/us/en/vehicle_protection_plan/guaranteed_auto_protection.html</t>
   </si>
   <si>
+    <t>us/en/vehicle-protection-plan/how-to-file-a-claim.report.json</t>
+  </si>
+  <si>
+    <t>["columns-callout","tabs-plans"]</t>
+  </si>
+  <si>
+    <t>us/en/vehicle-protection-plan/how-to-file-a-claim</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:16:49.792Z</t>
+  </si>
+  <si>
+    <t>How to File a Claim | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/vehicle_protection_plan/how_to_file_a_claim.html</t>
+  </si>
+  <si>
     <t>us/en/vehicle-protection-plan/prepaid-maintenance-plan.report.json</t>
   </si>
   <si>
@@ -421,6 +454,21 @@
     <t>https://www.toyotafinancial.com/us/en/vehicle_protection_plan/which_plan_is_right_for_me.html</t>
   </si>
   <si>
+    <t>us/en/financing-options/for-businesses/business-credit-applications.report.json</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/for-businesses/business-credit-applications</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:11:25.462Z</t>
+  </si>
+  <si>
+    <t>Business Credit Application | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/for_businesses/business_credit_applications.html</t>
+  </si>
+  <si>
     <t>us/en/financing-options/for-businesses/business-solutions.report.json</t>
   </si>
   <si>
@@ -439,6 +487,21 @@
     <t>https://www.toyotafinancial.com/us/en/financing_options/for_businesses/business_solutions.html</t>
   </si>
   <si>
+    <t>us/en/financing-options/rebate-finance-programs/college-rebate-program.report.json</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/rebate-finance-programs/college-rebate-program</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:11:14.381Z</t>
+  </si>
+  <si>
+    <t>College Rebate Program | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/rebate_finance_programs/college_rebate_program.html</t>
+  </si>
+  <si>
     <t>us/en/financing-options/rebate-finance-programs/find-rebate-finance-programs.report.json</t>
   </si>
   <si>
@@ -452,6 +515,21 @@
   </si>
   <si>
     <t>https://www.toyotafinancial.com/us/en/financing_options/rebate_finance_programs/find_rebate_finance_programs.html</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/rebate-finance-programs/military-rebate-program.report.json</t>
+  </si>
+  <si>
+    <t>us/en/financing-options/rebate-finance-programs/military-rebate-program</t>
+  </si>
+  <si>
+    <t>2026-10-04T06:11:19.736Z</t>
+  </si>
+  <si>
+    <t>Military Rebate Program | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/financing_options/rebate_finance_programs/military_rebate_program.html</t>
   </si>
   <si>
     <t>us/en/financing-options/rebate-finance-programs/repeat-customers.report.json</t>
@@ -1473,7 +1551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -1967,16 +2045,16 @@
         <v>100</v>
       </c>
       <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" t="s">
         <v>101</v>
-      </c>
-      <c r="C16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16" t="s">
-        <v>102</v>
       </c>
       <c r="F16" t="s">
         <v>14</v>
@@ -1985,30 +2063,30 @@
         <v>29</v>
       </c>
       <c r="H16" t="s">
+        <v>102</v>
+      </c>
+      <c r="I16" t="s">
         <v>103</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>104</v>
-      </c>
-      <c r="J16" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>105</v>
+      </c>
+      <c r="B17" t="s">
         <v>106</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
         <v>107</v>
-      </c>
-      <c r="C17" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" t="s">
-        <v>108</v>
       </c>
       <c r="F17" t="s">
         <v>14</v>
@@ -2017,30 +2095,30 @@
         <v>29</v>
       </c>
       <c r="H17" t="s">
+        <v>108</v>
+      </c>
+      <c r="I17" t="s">
         <v>109</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>110</v>
-      </c>
-      <c r="J17" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>111</v>
+      </c>
+      <c r="B18" t="s">
         <v>112</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
         <v>113</v>
-      </c>
-      <c r="C18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" t="s">
-        <v>114</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
@@ -2049,30 +2127,30 @@
         <v>29</v>
       </c>
       <c r="H18" t="s">
+        <v>114</v>
+      </c>
+      <c r="I18" t="s">
         <v>115</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>116</v>
-      </c>
-      <c r="J18" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" t="s">
         <v>118</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
         <v>119</v>
-      </c>
-      <c r="C19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" t="s">
-        <v>120</v>
       </c>
       <c r="F19" t="s">
         <v>14</v>
@@ -2081,30 +2159,30 @@
         <v>29</v>
       </c>
       <c r="H19" t="s">
+        <v>120</v>
+      </c>
+      <c r="I19" t="s">
         <v>121</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>122</v>
-      </c>
-      <c r="J19" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>123</v>
+      </c>
+      <c r="B20" t="s">
         <v>124</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
         <v>125</v>
-      </c>
-      <c r="C20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" t="s">
-        <v>126</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
@@ -2113,30 +2191,30 @@
         <v>29</v>
       </c>
       <c r="H20" t="s">
+        <v>126</v>
+      </c>
+      <c r="I20" t="s">
         <v>127</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>128</v>
-      </c>
-      <c r="J20" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" t="s">
         <v>130</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" t="s">
         <v>131</v>
-      </c>
-      <c r="C21" t="s">
-        <v>12</v>
-      </c>
-      <c r="D21" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" t="s">
-        <v>132</v>
       </c>
       <c r="F21" t="s">
         <v>14</v>
@@ -2145,30 +2223,30 @@
         <v>29</v>
       </c>
       <c r="H21" t="s">
+        <v>132</v>
+      </c>
+      <c r="I21" t="s">
         <v>133</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>134</v>
-      </c>
-      <c r="J21" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>135</v>
+      </c>
+      <c r="B22" t="s">
         <v>136</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" t="s">
         <v>137</v>
-      </c>
-      <c r="C22" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" t="s">
-        <v>138</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
@@ -2177,21 +2255,21 @@
         <v>29</v>
       </c>
       <c r="H22" t="s">
+        <v>138</v>
+      </c>
+      <c r="I22" t="s">
         <v>139</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>140</v>
-      </c>
-      <c r="J22" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>141</v>
+      </c>
+      <c r="B23" t="s">
         <v>142</v>
-      </c>
-      <c r="B23" t="s">
-        <v>69</v>
       </c>
       <c r="C23" t="s">
         <v>12</v>
@@ -2223,7 +2301,7 @@
         <v>147</v>
       </c>
       <c r="B24" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
@@ -2255,7 +2333,7 @@
         <v>152</v>
       </c>
       <c r="B25" t="s">
-        <v>27</v>
+        <v>153</v>
       </c>
       <c r="C25" t="s">
         <v>12</v>
@@ -2264,7 +2342,7 @@
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F25" t="s">
         <v>14</v>
@@ -2273,21 +2351,21 @@
         <v>29</v>
       </c>
       <c r="H25" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I25" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J25" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B26" t="s">
-        <v>27</v>
+        <v>69</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
@@ -2296,7 +2374,7 @@
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F26" t="s">
         <v>14</v>
@@ -2305,21 +2383,21 @@
         <v>29</v>
       </c>
       <c r="H26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I26" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J26" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B27" t="s">
-        <v>163</v>
+        <v>69</v>
       </c>
       <c r="C27" t="s">
         <v>12</v>
@@ -2334,152 +2412,152 @@
         <v>14</v>
       </c>
       <c r="G27" t="s">
+        <v>29</v>
+      </c>
+      <c r="H27" t="s">
         <v>165</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>166</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>167</v>
-      </c>
-      <c r="J27" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>168</v>
+      </c>
+      <c r="B28" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
         <v>169</v>
       </c>
-      <c r="B28" t="s">
-        <v>163</v>
-      </c>
-      <c r="C28" t="s">
-        <v>12</v>
-      </c>
-      <c r="D28" t="s">
-        <v>12</v>
-      </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>29</v>
+      </c>
+      <c r="H28" t="s">
         <v>170</v>
       </c>
-      <c r="F28" t="s">
-        <v>14</v>
-      </c>
-      <c r="G28" t="s">
-        <v>165</v>
-      </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>171</v>
       </c>
-      <c r="I28" t="s">
+      <c r="J28" t="s">
         <v>172</v>
-      </c>
-      <c r="J28" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>173</v>
+      </c>
+      <c r="B29" t="s">
+        <v>69</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
         <v>174</v>
       </c>
-      <c r="B29" t="s">
-        <v>163</v>
-      </c>
-      <c r="C29" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>29</v>
+      </c>
+      <c r="H29" t="s">
         <v>175</v>
       </c>
-      <c r="F29" t="s">
-        <v>14</v>
-      </c>
-      <c r="G29" t="s">
-        <v>165</v>
-      </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>176</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>177</v>
-      </c>
-      <c r="J29" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>178</v>
+      </c>
+      <c r="B30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" t="s">
         <v>179</v>
       </c>
-      <c r="B30" t="s">
-        <v>163</v>
-      </c>
-      <c r="C30" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" t="s">
+        <v>29</v>
+      </c>
+      <c r="H30" t="s">
         <v>180</v>
       </c>
-      <c r="F30" t="s">
-        <v>14</v>
-      </c>
-      <c r="G30" t="s">
-        <v>165</v>
-      </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>181</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>182</v>
-      </c>
-      <c r="J30" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>183</v>
+      </c>
+      <c r="B31" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" t="s">
         <v>184</v>
       </c>
-      <c r="B31" t="s">
-        <v>163</v>
-      </c>
-      <c r="C31" t="s">
-        <v>12</v>
-      </c>
-      <c r="D31" t="s">
-        <v>12</v>
-      </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" t="s">
+        <v>29</v>
+      </c>
+      <c r="H31" t="s">
         <v>185</v>
       </c>
-      <c r="F31" t="s">
-        <v>14</v>
-      </c>
-      <c r="G31" t="s">
-        <v>165</v>
-      </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>186</v>
       </c>
-      <c r="I31" t="s">
+      <c r="J31" t="s">
         <v>187</v>
-      </c>
-      <c r="J31" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>188</v>
+      </c>
+      <c r="B32" t="s">
         <v>189</v>
-      </c>
-      <c r="B32" t="s">
-        <v>163</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
@@ -2494,24 +2572,24 @@
         <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H32" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I32" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J32" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B33" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C33" t="s">
         <v>12</v>
@@ -2520,30 +2598,30 @@
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F33" t="s">
         <v>14</v>
       </c>
       <c r="G33" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H33" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I33" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J33" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B34" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C34" t="s">
         <v>12</v>
@@ -2552,30 +2630,30 @@
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F34" t="s">
         <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H34" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I34" t="s">
-        <v>140</v>
+        <v>203</v>
       </c>
       <c r="J34" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B35" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C35" t="s">
         <v>12</v>
@@ -2584,30 +2662,30 @@
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F35" t="s">
         <v>14</v>
       </c>
       <c r="G35" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H35" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I35" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="J35" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B36" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C36" t="s">
         <v>12</v>
@@ -2616,30 +2694,30 @@
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F36" t="s">
         <v>14</v>
       </c>
       <c r="G36" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H36" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="I36" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="J36" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B37" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C37" t="s">
         <v>12</v>
@@ -2648,30 +2726,30 @@
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F37" t="s">
         <v>14</v>
       </c>
       <c r="G37" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H37" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I37" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="J37" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B38" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C38" t="s">
         <v>12</v>
@@ -2680,30 +2758,30 @@
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F38" t="s">
         <v>14</v>
       </c>
       <c r="G38" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H38" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I38" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J38" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B39" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C39" t="s">
         <v>12</v>
@@ -2712,30 +2790,30 @@
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F39" t="s">
         <v>14</v>
       </c>
       <c r="G39" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H39" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I39" t="s">
-        <v>226</v>
+        <v>156</v>
       </c>
       <c r="J39" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B40" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C40" t="s">
         <v>12</v>
@@ -2744,30 +2822,30 @@
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F40" t="s">
         <v>14</v>
       </c>
       <c r="G40" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H40" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I40" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J40" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B41" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C41" t="s">
         <v>12</v>
@@ -2776,30 +2854,30 @@
         <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F41" t="s">
         <v>14</v>
       </c>
       <c r="G41" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H41" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I41" t="s">
-        <v>128</v>
+        <v>237</v>
       </c>
       <c r="J41" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B42" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C42" t="s">
         <v>12</v>
@@ -2808,30 +2886,30 @@
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F42" t="s">
         <v>14</v>
       </c>
       <c r="G42" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H42" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="I42" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="J42" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B43" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C43" t="s">
         <v>12</v>
@@ -2840,30 +2918,30 @@
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F43" t="s">
         <v>14</v>
       </c>
       <c r="G43" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H43" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I43" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="J43" t="s">
-        <v>79</v>
+        <v>248</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B44" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C44" t="s">
         <v>12</v>
@@ -2872,30 +2950,30 @@
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F44" t="s">
         <v>14</v>
       </c>
       <c r="G44" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H44" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="I44" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="J44" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B45" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C45" t="s">
         <v>12</v>
@@ -2904,30 +2982,30 @@
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="F45" t="s">
         <v>14</v>
       </c>
       <c r="G45" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H45" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="I45" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="J45" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B46" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C46" t="s">
         <v>12</v>
@@ -2936,30 +3014,30 @@
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="F46" t="s">
         <v>14</v>
       </c>
       <c r="G46" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H46" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="I46" t="s">
-        <v>259</v>
+        <v>139</v>
       </c>
       <c r="J46" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B47" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C47" t="s">
         <v>12</v>
@@ -2968,30 +3046,30 @@
         <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F47" t="s">
         <v>14</v>
       </c>
       <c r="G47" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H47" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="I47" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="J47" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B48" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C48" t="s">
         <v>12</v>
@@ -3000,30 +3078,30 @@
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F48" t="s">
         <v>14</v>
       </c>
       <c r="G48" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H48" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="I48" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="J48" t="s">
-        <v>270</v>
+        <v>79</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B49" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C49" t="s">
         <v>12</v>
@@ -3032,30 +3110,30 @@
         <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F49" t="s">
         <v>14</v>
       </c>
       <c r="G49" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H49" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="I49" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J49" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B50" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C50" t="s">
         <v>12</v>
@@ -3064,30 +3142,30 @@
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F50" t="s">
         <v>14</v>
       </c>
       <c r="G50" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H50" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="I50" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J50" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B51" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C51" t="s">
         <v>12</v>
@@ -3096,30 +3174,30 @@
         <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F51" t="s">
         <v>14</v>
       </c>
       <c r="G51" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H51" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I51" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J51" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B52" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C52" t="s">
         <v>12</v>
@@ -3128,30 +3206,30 @@
         <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F52" t="s">
         <v>14</v>
       </c>
       <c r="G52" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H52" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I52" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J52" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B53" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C53" t="s">
         <v>12</v>
@@ -3160,30 +3238,30 @@
         <v>12</v>
       </c>
       <c r="E53" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F53" t="s">
         <v>14</v>
       </c>
       <c r="G53" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H53" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="I53" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J53" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B54" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C54" t="s">
         <v>12</v>
@@ -3192,30 +3270,30 @@
         <v>12</v>
       </c>
       <c r="E54" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F54" t="s">
         <v>14</v>
       </c>
       <c r="G54" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H54" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="I54" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J54" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B55" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C55" t="s">
         <v>12</v>
@@ -3224,30 +3302,30 @@
         <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F55" t="s">
         <v>14</v>
       </c>
       <c r="G55" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H55" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I55" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J55" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B56" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C56" t="s">
         <v>12</v>
@@ -3256,30 +3334,30 @@
         <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F56" t="s">
         <v>14</v>
       </c>
       <c r="G56" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H56" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="I56" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J56" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B57" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C57" t="s">
         <v>12</v>
@@ -3288,30 +3366,30 @@
         <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F57" t="s">
         <v>14</v>
       </c>
       <c r="G57" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H57" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="I57" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J57" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B58" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C58" t="s">
         <v>12</v>
@@ -3320,30 +3398,30 @@
         <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F58" t="s">
         <v>14</v>
       </c>
       <c r="G58" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H58" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="I58" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J58" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B59" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C59" t="s">
         <v>12</v>
@@ -3352,30 +3430,30 @@
         <v>12</v>
       </c>
       <c r="E59" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F59" t="s">
         <v>14</v>
       </c>
       <c r="G59" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H59" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="I59" t="s">
-        <v>150</v>
+        <v>325</v>
       </c>
       <c r="J59" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B60" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C60" t="s">
         <v>12</v>
@@ -3384,30 +3462,30 @@
         <v>12</v>
       </c>
       <c r="E60" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="F60" t="s">
         <v>14</v>
       </c>
       <c r="G60" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H60" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="I60" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="J60" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B61" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C61" t="s">
         <v>12</v>
@@ -3416,30 +3494,30 @@
         <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="F61" t="s">
         <v>14</v>
       </c>
       <c r="G61" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H61" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="I61" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="J61" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B62" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C62" t="s">
         <v>12</v>
@@ -3448,30 +3526,30 @@
         <v>12</v>
       </c>
       <c r="E62" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F62" t="s">
         <v>14</v>
       </c>
       <c r="G62" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H62" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="I62" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="J62" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B63" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C63" t="s">
         <v>12</v>
@@ -3480,30 +3558,30 @@
         <v>12</v>
       </c>
       <c r="E63" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="F63" t="s">
         <v>14</v>
       </c>
       <c r="G63" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H63" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="I63" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="J63" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B64" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C64" t="s">
         <v>12</v>
@@ -3512,54 +3590,214 @@
         <v>12</v>
       </c>
       <c r="E64" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="F64" t="s">
         <v>14</v>
       </c>
       <c r="G64" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="H64" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="I64" t="s">
-        <v>348</v>
+        <v>176</v>
       </c>
       <c r="J64" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B65" t="s">
-        <v>12</v>
+        <v>189</v>
       </c>
       <c r="C65" t="s">
-        <v>351</v>
+        <v>12</v>
       </c>
       <c r="D65" t="s">
+        <v>12</v>
+      </c>
+      <c r="E65" t="s">
         <v>352</v>
       </c>
-      <c r="E65" t="s">
+      <c r="F65" t="s">
+        <v>14</v>
+      </c>
+      <c r="G65" t="s">
+        <v>191</v>
+      </c>
+      <c r="H65" t="s">
         <v>353</v>
       </c>
-      <c r="F65" t="s">
+      <c r="I65" t="s">
         <v>354</v>
       </c>
-      <c r="G65" t="s">
-        <v>12</v>
-      </c>
-      <c r="H65" t="s">
+      <c r="J65" t="s">
         <v>355</v>
       </c>
-      <c r="I65" t="s">
-        <v>12</v>
-      </c>
-      <c r="J65" t="s">
-        <v>168</v>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>356</v>
+      </c>
+      <c r="B66" t="s">
+        <v>189</v>
+      </c>
+      <c r="C66" t="s">
+        <v>12</v>
+      </c>
+      <c r="D66" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" t="s">
+        <v>357</v>
+      </c>
+      <c r="F66" t="s">
+        <v>14</v>
+      </c>
+      <c r="G66" t="s">
+        <v>191</v>
+      </c>
+      <c r="H66" t="s">
+        <v>358</v>
+      </c>
+      <c r="I66" t="s">
+        <v>359</v>
+      </c>
+      <c r="J66" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>361</v>
+      </c>
+      <c r="B67" t="s">
+        <v>189</v>
+      </c>
+      <c r="C67" t="s">
+        <v>12</v>
+      </c>
+      <c r="D67" t="s">
+        <v>12</v>
+      </c>
+      <c r="E67" t="s">
+        <v>362</v>
+      </c>
+      <c r="F67" t="s">
+        <v>14</v>
+      </c>
+      <c r="G67" t="s">
+        <v>191</v>
+      </c>
+      <c r="H67" t="s">
+        <v>363</v>
+      </c>
+      <c r="I67" t="s">
+        <v>364</v>
+      </c>
+      <c r="J67" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>366</v>
+      </c>
+      <c r="B68" t="s">
+        <v>189</v>
+      </c>
+      <c r="C68" t="s">
+        <v>12</v>
+      </c>
+      <c r="D68" t="s">
+        <v>12</v>
+      </c>
+      <c r="E68" t="s">
+        <v>367</v>
+      </c>
+      <c r="F68" t="s">
+        <v>14</v>
+      </c>
+      <c r="G68" t="s">
+        <v>191</v>
+      </c>
+      <c r="H68" t="s">
+        <v>368</v>
+      </c>
+      <c r="I68" t="s">
+        <v>369</v>
+      </c>
+      <c r="J68" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>371</v>
+      </c>
+      <c r="B69" t="s">
+        <v>189</v>
+      </c>
+      <c r="C69" t="s">
+        <v>12</v>
+      </c>
+      <c r="D69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69" t="s">
+        <v>372</v>
+      </c>
+      <c r="F69" t="s">
+        <v>14</v>
+      </c>
+      <c r="G69" t="s">
+        <v>191</v>
+      </c>
+      <c r="H69" t="s">
+        <v>373</v>
+      </c>
+      <c r="I69" t="s">
+        <v>374</v>
+      </c>
+      <c r="J69" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>376</v>
+      </c>
+      <c r="B70" t="s">
+        <v>12</v>
+      </c>
+      <c r="C70" t="s">
+        <v>377</v>
+      </c>
+      <c r="D70" t="s">
+        <v>378</v>
+      </c>
+      <c r="E70" t="s">
+        <v>379</v>
+      </c>
+      <c r="F70" t="s">
+        <v>380</v>
+      </c>
+      <c r="G70" t="s">
+        <v>12</v>
+      </c>
+      <c r="H70" t="s">
+        <v>381</v>
+      </c>
+      <c r="I70" t="s">
+        <v>12</v>
+      </c>
+      <c r="J70" t="s">
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>